<commit_message>
docs: make sure bom and schematics are consistent
Update bill of material to make sure it is consistent
with the current version of the schematics. Re-export
schematics for good measure as well.

Signed-off-by: Stefan Gloor <code@stefan-gloor.ch>
</commit_message>
<xml_diff>
--- a/docs/bom/bom.xlsx
+++ b/docs/bom/bom.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
   <si>
     <t xml:space="preserve">Bill of Materials (BOM)</t>
   </si>
@@ -34,6 +34,9 @@
     <t xml:space="preserve">Date:</t>
   </si>
   <si>
+    <t xml:space="preserve">22.7.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
@@ -82,22 +85,30 @@
     <t xml:space="preserve">C2922443</t>
   </si>
   <si>
-    <t xml:space="preserve">Q1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Package_TO_SOT_SMD:SOT-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toshiba Semiconductor and Storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SSM3K344R,LF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digikey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SSM3K344RLFTR-ND</t>
+    <t xml:space="preserve">For use with adapter board
+Better use compatible straddle
+Mount type, e.g., from LOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOT23-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas Instruments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TLV71211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mouser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">595-TLV71211DBVR</t>
   </si>
   <si>
     <t xml:space="preserve">D1</t>
@@ -109,40 +120,16 @@
     <t xml:space="preserve">LED_SMD:LED_0805_2012Metric</t>
   </si>
   <si>
-    <t xml:space="preserve">Kingbright</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APHCM2012CGCK-F01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">754-1094-2-ND</t>
+    <t xml:space="preserve">generic</t>
   </si>
   <si>
     <t xml:space="preserve">R1</t>
   </si>
   <si>
-    <t xml:space="preserve">10k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do Not Populate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Resistor_SMD:R_0603_1608Metric</t>
   </si>
   <si>
-    <t xml:space="preserve">Bourns Inc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CR0603-JW-331ELF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CR0603-JW-331ELFTR-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1,C2,C3,C4</t>
+    <t xml:space="preserve">C1,C3</t>
   </si>
   <si>
     <t xml:space="preserve">100n</t>
@@ -151,15 +138,6 @@
     <t xml:space="preserve">Capacitor_SMD:C_0603_1608Metric</t>
   </si>
   <si>
-    <t xml:space="preserve">Samsung Electro-Mechanics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CL10B104KB8NNWC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1276-1935-2-ND</t>
-  </si>
-  <si>
     <t xml:space="preserve">J1</t>
   </si>
   <si>
@@ -172,34 +150,43 @@
     <t xml:space="preserve">501951-2430</t>
   </si>
   <si>
-    <t xml:space="preserve">Mouser</t>
-  </si>
-  <si>
     <t xml:space="preserve">    538-501951-2430</t>
   </si>
   <si>
-    <t xml:space="preserve">C5</t>
+    <t xml:space="preserve">C2</t>
   </si>
   <si>
     <t xml:space="preserve">2.2u</t>
   </si>
   <si>
-    <t xml:space="preserve">CL10A225KO8NNNC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1276-1040-2-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U3-U9</t>
+    <t xml:space="preserve">U4-U12,
+U22-U27,
+U33,U35</t>
   </si>
   <si>
     <t xml:space="preserve">ddr5:STQFN-12LD-0.5</t>
   </si>
   <si>
-    <t xml:space="preserve">MACOM Technology Solutions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MASW-009482-TR3000</t>
+    <t xml:space="preserve">TMUX136</t>
+  </si>
+  <si>
+    <t xml:space="preserve">595-TMUX136MRSER </t>
+  </si>
+  <si>
+    <t xml:space="preserve">U13-U21,
+U28-U32,U34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOT-363-6 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diodes Inc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PI5A3157CEX </t>
+  </si>
+  <si>
+    <t xml:space="preserve">729-PI5A3157CEX </t>
   </si>
 </sst>
 </file>
@@ -210,7 +197,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -241,13 +228,6 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF666666"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -328,7 +308,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -340,15 +320,15 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -409,7 +389,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666666"/>
+      <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -424,13 +404,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18A303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369A3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A33E03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8E03A3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="C99C00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="C9211E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000EE"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551A8B"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.55"/>
@@ -441,7 +527,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="31.3"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="29.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -490,8 +576,8 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>44992</v>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -516,37 +602,37 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>1</v>
       </c>
@@ -554,25 +640,27 @@
         <v>1</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="J7" s="7"/>
+        <v>20</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
@@ -582,23 +670,25 @@
         <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="7"/>
+        <v>22</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="E8" s="7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>28</v>
       </c>
       <c r="J8" s="7"/>
     </row>
@@ -610,77 +700,85 @@
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J9" s="7"/>
     </row>
-    <row r="10" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8" t="s">
+      <c r="D10" s="7" t="n">
+        <v>330</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="F10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="7" t="n">
-        <v>330</v>
+      <c r="D11" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="J11" s="7"/>
     </row>
@@ -689,28 +787,26 @@
         <v>6</v>
       </c>
       <c r="B12" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="H12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>45</v>
       </c>
       <c r="J12" s="7"/>
     </row>
@@ -722,81 +818,81 @@
         <v>1</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="7"/>
+        <v>43</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>44</v>
+      </c>
       <c r="E13" s="7" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>51</v>
+        <v>32</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="J13" s="7"/>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>53</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="7"/>
       <c r="E14" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>55</v>
+        <v>27</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="J14" s="7"/>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>56</v>
+        <v>15</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="D15" s="7"/>
-      <c r="E15" s="7" t="s">
-        <v>57</v>
+      <c r="E15" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>59</v>
+        <v>51</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>59</v>
+        <v>27</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="J15" s="7"/>
     </row>
@@ -883,18 +979,6 @@
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
       <c r="J22" s="7"/>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>